<commit_message>
diário: validação do ambiente Docker em 24/09
</commit_message>
<xml_diff>
--- a/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
+++ b/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,70 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Validação do Saborino via Docker no Mac (forma A): build das imagens, migrate, seed fictício, smoke da API e da tela inicial, e encerramento dos containers. Problemas encontrados e corrigidos: o helper de credenciais do Docker estava fora do PATH; o script de smoke não funcionava no bash 3.2 do macOS (a 1ª tentativa foi mantida como registro); e uma 1ª chamada do script de migrate falhou no shell antes de executar qualquer comando do Docker e foi refeita.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>01_SISTEMA_ALVO/evidencias_ambiente/2026-09-24_docker_*.txt; 01_SISTEMA_ALVO/ambiente_p2/smoke_api.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Atualização do README (pasta 00) com os comandos validados da forma A e os problemas conhecidos do ambiente Mac</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>00_IDENTIFICACAO_E_README/README.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
diário: anonimização antes da publicação em 24/09
</commit_message>
<xml_diff>
--- a/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
+++ b/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -509,7 +509,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>00_IDENTIFICACAO_E_README/P01_FICHA_PROPOSTA_SISTEMA_v0.1.pdf</t>
+          <t>00_IDENTIFICACAO_E_README/P01_FICHA_PROPOSTA_SISTEMA_v0.2.docx (a v0.1 foi retirada na anonimização de 24/09)</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>00_IDENTIFICACAO_E_README/README.md; RESUMO_ANDAMENTO_2026-09-24.pdf</t>
+          <t>00_IDENTIFICACAO_E_README/README.md; RESUMO_ANDAMENTO_2026-09-24_v0.2.docx (a v0.1 foi retirada na anonimização de 24/09)</t>
         </is>
       </c>
     </row>
@@ -702,6 +702,38 @@
       <c r="F10" s="3" t="inlineStr">
         <is>
           <t>00_IDENTIFICACAO_E_README/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Anonimização antes da publicação no GitHub: retirada dos arquivos de implantação e operação de ambientes reais; troca dos dados padrão que identificavam o uso real por valores neutros; nova versão neutra (v0.2) da Ficha A e do resumo de andamento; e reescrita do histórico do repositório para que nenhuma versão anterior exponha essas informações. Exceção registrada à regra de versões da seção 7: as v0.1 da Ficha e do resumo saíram do histórico por conterem informações do uso real. Revalidação: 69 testes do backend, migrate e seed num banco novo, smoke da API, Vitest e build do frontend.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>01_SISTEMA_ALVO/DESVIOS_DA_RELEASE.md; 01_SISTEMA_ALVO/evidencias_ambiente/2026-09-24_docker_validacao_codigo_anonimizado.txt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
diário: publicação do repositório em 24/09
</commit_message>
<xml_diff>
--- a/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
+++ b/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -737,6 +737,38 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Criação do repositório público no GitHub e primeiro push, depois da varredura de todo o histórico (nenhuma ocorrência dos termos sensíveis)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/LeonardoVDN/P2_TQS_2026_CC_GRUPO13_SABORINO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
diário: documentos v0.3 para a aula de 24/09
</commit_message>
<xml_diff>
--- a/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
+++ b/15_DIARIO_DE_PARTICIPACAO/DIARIO_DE_PARTICIPACAO.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -769,6 +769,38 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Ficha do Apêndice A e resumo de andamento v0.3 para a aula: link do repositório, execução via Docker, evidências de 24/09 e próximos passos atualizados</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>[a preencher pelo grupo]</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>00_IDENTIFICACAO_E_README/P01_FICHA_PROPOSTA_SISTEMA_v0.3.pdf; RESUMO_ANDAMENTO_2026-09-24_v0.3.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>